<commit_message>
recrated some of the descriptions from derivedFrom
</commit_message>
<xml_diff>
--- a/output/all-profiles.xlsx
+++ b/output/all-profiles.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-07-27T11:31:10-04:00</t>
+    <t>2025-07-27T11:33:37-04:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1607,7 +1607,7 @@
     <t>(USCDI) US Core Profiles or other resource the observation is made from</t>
   </si>
   <si>
-    <t>Observations or or other resource such as a QuestionnaireResponse from which this observation value is derived.</t>
+    <t>Observations from which this observation value is derived.</t>
   </si>
   <si>
     <t>All the reference choices that are listed in this element can represent clinical observations and other measurements that may be the source for a derived value.  The most common reference will be another Observation.  For a discussion on the ways Observations can assembled in groups together, see [Notes](http://hl7.org/fhir/R4/observation.html#obsgrouping) below.</t>

</xml_diff>

<commit_message>
commit before trying gofsh generated file
</commit_message>
<xml_diff>
--- a/output/all-profiles.xlsx
+++ b/output/all-profiles.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-07-27T11:33:37-04:00</t>
+    <t>2025-07-27T15:07:55-04:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -9401,7 +9401,7 @@
       </c>
       <c r="F69" s="2"/>
       <c r="G69" t="s" s="2">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="H69" t="s" s="2">
         <v>81</v>

</xml_diff>